<commit_message>
Worst-Case-Einzelsonden reproduzierbar, Oracle-Gap quantifiziert, Analyse-Dokument, englischer Einstieg
- sbench.probe_study: Einzelsonden-Test (7 statt 32 Auswertungen) für die drei ODD-Probleme, mit Test
- sbench.oracle_gap: Anteil der mit Plattform-Bremsgrenze unvermeidbaren 'gültigen' Fehler
- docs/Kritische_Szenarien_L4-Shuttle.md: Konzept, Ergebnisse, Abgleich Stand/Gaps/Fragen
- Excel um Blatt 'Gaps zum echten System' ergänzt, README mit englischer Übersicht, MIT-Lizenz

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results_suite/Sensormodelle_Gesamtkette_Abdeckung.xlsx
+++ b/results_suite/Sensormodelle_Gesamtkette_Abdeckung.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budgets Rueckrechnung" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reichweite Stehendes Hindernis" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annahmen Stufe 1" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gaps zum echten System" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sensor x Stufe'!$A$1:$E$9</definedName>
@@ -5216,4 +5217,421 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Stand im Bench</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Risiko ggü. echtem System</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Maßnahme</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Priorität</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Sicherheit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Orakel für „vermeidbar“</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Bremst mit µ·g (bis ca. 9 m/s²), Shuttle ist auf 4 bzw. 6 m/s² ausgelegt</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Physikalisch unvermeidbare Fälle zählen als gültige Fehler, P_f zu hoch</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Orakel auf Bremsgrenze der Plattform begrenzen, ATS-Läufe neu rechnen</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>1 (zuerst)</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Wahrscheinlich</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Common-Cause statt unabhängiger Sensorfehler</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Fehler je Scan und Sensor unabhängig</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Regen, Gegenlicht, Verschmutzung treffen mehrere Sensoren gleichzeitig; 0 % bei Radar+X vermutlich Artefakt</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Variante mit korrelierten Ausfällen, Redundanzgewinn neu messen</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Wahrscheinlich</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Fusion und Tracker</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Minimum der Sensoren, kein Tracker</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Bestätigungszeit, Track-Verlust, ID-Wechsel, Prädiktion beeinflussen Phantombremsen und Cut-in</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Tracker-Modell oder echte Tracker-Software einbinden, 2-aus-3-Fusion testen</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Wahrscheinlich</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Latenz als Konstante</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Feste Latenz plus Jitter bis 0,05 s; dominiert in 85–98 % der Fälle</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Reale Latenz: Verteilungen je Stufe mit schweren Rändern (Scheduling, GPU-Last, Zeitstempel, Uhrensync)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Latenzen messen, auf Tails/WCET auslegen</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Dominanz wahrscheinlich, Form Vermutung</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Aktorik und Severity</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Verzögerungsglied 1. Ordnung, Reibgrenze, Schaden nur über Aufprallgeschwindigkeit</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Totzeit, Druckaufbau, Hysterese, Rekuperation, ABS fehlen; Verletzungsgefahr stehender Fahrgäste fehlt</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Bremsmodell mit Totzeit/Rampe, zweites Schadensmaß</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Vermutung</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Szenarien, ODD, Prior</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>1D-Längsdynamik, Fußgänger geradlinig mit konstanter Geschwindigkeit, erfundene Beta-Priors</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Gruppen, Kinder, Rollstühle, Intentionswechsel, Radfahrer, Mischverkehr fehlen; P_f keine Risikozahl</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>ODD formal beschreiben, Expositionsdaten vom Betriebsort</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Vermutung</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Weltmodell und Lokalisierung</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Ein Entfernungswert pro Sensor, Umgebung als Reichweitenfaktor</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Freiraum, Belegungskarte, Eigenlokalisierung fehlen</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Belegungsmodell, Lokalisierungsfehler als Abweichung</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Vermutung</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>FMUs für echte Software</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Python-Simulation, ca. 7 ms pro Lauf</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Echte Software wohl 100–1000× langsamer; Reproduzierbarkeit braucht feste Schrittweite und Seeds</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Wenige Validierungsläufe mit echter SW, Suche über Vorabschätzung/Surrogat</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Vermutung</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Netzwerk</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Latenz, Jitter, Verlust</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Für Stufe 1 ausreichend, wenn Schranke konservativ</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Beibehalten, später Network Calculus</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>8 (niedrig)</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Vermutung</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Validierung des Modells</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Alle Parameter sind Annahmen</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Ohne Messdaten keine belastbare Aussage über das echte Shuttle</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Credibility-Bewertung, Parameter aus Messdaten, Gegenprobe gegen FAU/fiveD</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>begleitend</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Wahrscheinlich</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sicherheit: Wahrscheinlich = im Bench gestützt, aber unter Annahmen; Vermutung = Erfahrungswissen, nicht recherchiert.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>